<commit_message>
SS25 syllabus and other small updates
</commit_message>
<xml_diff>
--- a/files/CR_Publications.xlsx
+++ b/files/CR_Publications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rauh\NextCloudSync\WZB_CR\Datensaetze\ChRauh.github.io\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05B378FC-4E2C-4021-A739-523AF2B95F28}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75E1DBCB-2C45-4822-A3FC-2A39C0121464}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="592">
   <si>
     <t>Cites</t>
   </si>
@@ -1351,9 +1351,6 @@
     <t>10.17979/ejge.2013.2.1.4285</t>
   </si>
   <si>
-    <t>Online First</t>
-  </si>
-  <si>
     <t>https://www.tandfonline.com/doi/epdf/10.1080/01402382.2011.616659?needAccess=true</t>
   </si>
   <si>
@@ -1772,6 +1769,33 @@
   </si>
   <si>
     <t>doi:10.7910/DVN/L4OAKN</t>
+  </si>
+  <si>
+    <t>2025-07-15</t>
+  </si>
+  <si>
+    <t>51(5): 792-821</t>
+  </si>
+  <si>
+    <t>2025-09-30</t>
+  </si>
+  <si>
+    <t>2025</t>
+  </si>
+  <si>
+    <t>&lt;u&gt;Christian Rauh&lt;/u&gt;, Milan Schröder</t>
+  </si>
+  <si>
+    <t>189: 36-40</t>
+  </si>
+  <si>
+    <t>https://www.wzb.eu/de/publikationen/wzb-mitteilungen/nr-189-weltordnung</t>
+  </si>
+  <si>
+    <t>https://bibliothek.wzb.eu/artikel/2025/f-27188.pdf</t>
+  </si>
+  <si>
+    <t>**Zwischen Wirtschaft und Werten: Zum Selbst- und Fremdbild der Europäischen Union in der internationalen Ordnung**</t>
   </si>
 </sst>
 </file>
@@ -3184,6 +3208,314 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="AutoShape 3" descr="data:image/svg+xml;base64,PD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiPz48IURPQ1RZUEUgc3ZnIFBVQkxJQyAiLS8vVzNDLy9EVEQgU1ZHIDEuMS8vRU4iICJodHRwOi8vd3d3LnczLm9yZy9HcmFwaGljcy9TVkcvMS4xL0RURC9zdmcxMS5kdGQiPjxzdmcgdmVyc2lvbj0iMS4xIiBpZD0iRWJlbmVfMSIgeG1sbnM9Imh0dHA6Ly93d3cudzMub3JnLzIwMDAvc3ZnIiB4bWxuczp4bGluaz0iaHR0cDovL3d3dy53My5vcmcvMTk5OS94bGluayIgeD0iMHB4IiB5PSIwcHgiIHdpZHRoPSIxNnB4IiBoZWlnaHQ9IjE2cHgiIHZpZXdCb3g9IjAgMCAxNiAxNiIgZW5hYmxlLWJhY2tncm91bmQ9Im5ldyAwIDAgMTYgMTYiIHhtbDpzcGFjZT0icHJlc2VydmUiPjxnPjxnPjxwYXRoIGZpbGw9IiNGRkZGRkYiIGQ9Ik04LjAwMSwxNS41QzMuODY0LDE1LjUsMC41LDEyLjEzNiwwLjUsOGMwLTQuMTM1LDMuMzY1LTcuNSw3LjUwMS03LjVTMTUuNSwzLjg2NCwxNS41LDhTMTIuMTM3LDE1LjUsOC4wMDEsMTUuNXoiLz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNOC4wMDEsMUMxMS44NiwxLDE1LDQuMTQxLDE1LDhzLTMuMTM5LDctNi45OTksN0M0LjE0LDE1LDEsMTEuODU5LDEsOFM0LjE0LDEsOC4wMDEsMSBNOC4wMDEsMEMzLjU4MiwwLDAsMy41ODIsMCw4czMuNTgyLDgsOC4wMDEsOEMxMi40MTgsMTYsMTYsMTIuNDE4LDE2LDhTMTIuNDE4LDAsOC4wMDEsMEw4LjAwMSwweiIvPjwvZz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNNi43NDUsMTIuNTg5Yy0wLjIyNywwLjEyMi0wLjQ5NywwLjI0Ny0wLjY4NCwwLjI0N2MtMC4zMTgsMC0wLjUwMS0wLjE2NC0wLjUwMS0wLjQ1MmMwLTAuMjA3LDAuMTQtMC4zNzUsMC41OTUtMC42MjJjMS41NDktMC45MDQsMi41OTQtMi4yNzIsMi41OTQtMy43MjFjMC0wLjgyNS0wLjIyNy0xLjExOS0wLjY4MS0xLjExOWMtMC4xMzUsMC0wLjMyLDAuMjE5LTAuNjM2LDAuMjE5SDcuMTU3QzYuMTAyLDcuMTQzLDUuMzMzLDYuMjY0LDUuMzMzLDUuMjNjMC0xLjE1MiwwLjk1OC0yLjAwNiwyLjI4LTIuMDA2YzEuNzc3LDAsMy4wNTMsMS4zNzMsMy4wNTMsMy40M0MxMC42NjYsOS4yMTUsOS4yMDMsMTEuMjcsNi43NDUsMTIuNTg5Ii8+PC9nPjwvc3ZnPg">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AC0E3EB9-E3C6-43BB-B223-19E9E498CED7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11239500" y="12954000"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="22" name="AutoShape 3" descr="data:image/svg+xml;base64,PD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiPz48IURPQ1RZUEUgc3ZnIFBVQkxJQyAiLS8vVzNDLy9EVEQgU1ZHIDEuMS8vRU4iICJodHRwOi8vd3d3LnczLm9yZy9HcmFwaGljcy9TVkcvMS4xL0RURC9zdmcxMS5kdGQiPjxzdmcgdmVyc2lvbj0iMS4xIiBpZD0iRWJlbmVfMSIgeG1sbnM9Imh0dHA6Ly93d3cudzMub3JnLzIwMDAvc3ZnIiB4bWxuczp4bGluaz0iaHR0cDovL3d3dy53My5vcmcvMTk5OS94bGluayIgeD0iMHB4IiB5PSIwcHgiIHdpZHRoPSIxNnB4IiBoZWlnaHQ9IjE2cHgiIHZpZXdCb3g9IjAgMCAxNiAxNiIgZW5hYmxlLWJhY2tncm91bmQ9Im5ldyAwIDAgMTYgMTYiIHhtbDpzcGFjZT0icHJlc2VydmUiPjxnPjxnPjxwYXRoIGZpbGw9IiNGRkZGRkYiIGQ9Ik04LjAwMSwxNS41QzMuODY0LDE1LjUsMC41LDEyLjEzNiwwLjUsOGMwLTQuMTM1LDMuMzY1LTcuNSw3LjUwMS03LjVTMTUuNSwzLjg2NCwxNS41LDhTMTIuMTM3LDE1LjUsOC4wMDEsMTUuNXoiLz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNOC4wMDEsMUMxMS44NiwxLDE1LDQuMTQxLDE1LDhzLTMuMTM5LDctNi45OTksN0M0LjE0LDE1LDEsMTEuODU5LDEsOFM0LjE0LDEsOC4wMDEsMSBNOC4wMDEsMEMzLjU4MiwwLDAsMy41ODIsMCw4czMuNTgyLDgsOC4wMDEsOEMxMi40MTgsMTYsMTYsMTIuNDE4LDE2LDhTMTIuNDE4LDAsOC4wMDEsMEw4LjAwMSwweiIvPjwvZz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNNi43NDUsMTIuNTg5Yy0wLjIyNywwLjEyMi0wLjQ5NywwLjI0Ny0wLjY4NCwwLjI0N2MtMC4zMTgsMC0wLjUwMS0wLjE2NC0wLjUwMS0wLjQ1MmMwLTAuMjA3LDAuMTQtMC4zNzUsMC41OTUtMC42MjJjMS41NDktMC45MDQsMi41OTQtMi4yNzIsMi41OTQtMy43MjFjMC0wLjgyNS0wLjIyNy0xLjExOS0wLjY4MS0xLjExOWMtMC4xMzUsMC0wLjMyLDAuMjE5LTAuNjM2LDAuMjE5SDcuMTU3QzYuMTAyLDcuMTQzLDUuMzMzLDYuMjY0LDUuMzMzLDUuMjNjMC0xLjE1MiwwLjk1OC0yLjAwNiwyLjI4LTIuMDA2YzEuNzc3LDAsMy4wNTMsMS4zNzMsMy4wNTMsMy40M0MxMC42NjYsOS4yMTUsOS4yMDMsMTEuMjcsNi43NDUsMTIuNTg5Ii8+PC9nPjwvc3ZnPg">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3EC12B60-55AA-40FF-AD37-2FAAB9F50237}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11239500" y="12954000"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="23" name="AutoShape 3" descr="data:image/svg+xml;base64,PD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiPz48IURPQ1RZUEUgc3ZnIFBVQkxJQyAiLS8vVzNDLy9EVEQgU1ZHIDEuMS8vRU4iICJodHRwOi8vd3d3LnczLm9yZy9HcmFwaGljcy9TVkcvMS4xL0RURC9zdmcxMS5kdGQiPjxzdmcgdmVyc2lvbj0iMS4xIiBpZD0iRWJlbmVfMSIgeG1sbnM9Imh0dHA6Ly93d3cudzMub3JnLzIwMDAvc3ZnIiB4bWxuczp4bGluaz0iaHR0cDovL3d3dy53My5vcmcvMTk5OS94bGluayIgeD0iMHB4IiB5PSIwcHgiIHdpZHRoPSIxNnB4IiBoZWlnaHQ9IjE2cHgiIHZpZXdCb3g9IjAgMCAxNiAxNiIgZW5hYmxlLWJhY2tncm91bmQ9Im5ldyAwIDAgMTYgMTYiIHhtbDpzcGFjZT0icHJlc2VydmUiPjxnPjxnPjxwYXRoIGZpbGw9IiNGRkZGRkYiIGQ9Ik04LjAwMSwxNS41QzMuODY0LDE1LjUsMC41LDEyLjEzNiwwLjUsOGMwLTQuMTM1LDMuMzY1LTcuNSw3LjUwMS03LjVTMTUuNSwzLjg2NCwxNS41LDhTMTIuMTM3LDE1LjUsOC4wMDEsMTUuNXoiLz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNOC4wMDEsMUMxMS44NiwxLDE1LDQuMTQxLDE1LDhzLTMuMTM5LDctNi45OTksN0M0LjE0LDE1LDEsMTEuODU5LDEsOFM0LjE0LDEsOC4wMDEsMSBNOC4wMDEsMEMzLjU4MiwwLDAsMy41ODIsMCw4czMuNTgyLDgsOC4wMDEsOEMxMi40MTgsMTYsMTYsMTIuNDE4LDE2LDhTMTIuNDE4LDAsOC4wMDEsMEw4LjAwMSwweiIvPjwvZz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNNi43NDUsMTIuNTg5Yy0wLjIyNywwLjEyMi0wLjQ5NywwLjI0Ny0wLjY4NCwwLjI0N2MtMC4zMTgsMC0wLjUwMS0wLjE2NC0wLjUwMS0wLjQ1MmMwLTAuMjA3LDAuMTQtMC4zNzUsMC41OTUtMC42MjJjMS41NDktMC45MDQsMi41OTQtMi4yNzIsMi41OTQtMy43MjFjMC0wLjgyNS0wLjIyNy0xLjExOS0wLjY4MS0xLjExOWMtMC4xMzUsMC0wLjMyLDAuMjE5LTAuNjM2LDAuMjE5SDcuMTU3QzYuMTAyLDcuMTQzLDUuMzMzLDYuMjY0LDUuMzMzLDUuMjNjMC0xLjE1MiwwLjk1OC0yLjAwNiwyLjI4LTIuMDA2YzEuNzc3LDAsMy4wNTMsMS4zNzMsMy4wNTMsMy40M0MxMC42NjYsOS4yMTUsOS4yMDMsMTEuMjcsNi43NDUsMTIuNTg5Ii8+PC9nPjwvc3ZnPg">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CAEED22A-1F48-4375-AFCA-A164EEFFC927}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11239500" y="12954000"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="24" name="AutoShape 3" descr="data:image/svg+xml;base64,PD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiPz48IURPQ1RZUEUgc3ZnIFBVQkxJQyAiLS8vVzNDLy9EVEQgU1ZHIDEuMS8vRU4iICJodHRwOi8vd3d3LnczLm9yZy9HcmFwaGljcy9TVkcvMS4xL0RURC9zdmcxMS5kdGQiPjxzdmcgdmVyc2lvbj0iMS4xIiBpZD0iRWJlbmVfMSIgeG1sbnM9Imh0dHA6Ly93d3cudzMub3JnLzIwMDAvc3ZnIiB4bWxuczp4bGluaz0iaHR0cDovL3d3dy53My5vcmcvMTk5OS94bGluayIgeD0iMHB4IiB5PSIwcHgiIHdpZHRoPSIxNnB4IiBoZWlnaHQ9IjE2cHgiIHZpZXdCb3g9IjAgMCAxNiAxNiIgZW5hYmxlLWJhY2tncm91bmQ9Im5ldyAwIDAgMTYgMTYiIHhtbDpzcGFjZT0icHJlc2VydmUiPjxnPjxnPjxwYXRoIGZpbGw9IiNGRkZGRkYiIGQ9Ik04LjAwMSwxNS41QzMuODY0LDE1LjUsMC41LDEyLjEzNiwwLjUsOGMwLTQuMTM1LDMuMzY1LTcuNSw3LjUwMS03LjVTMTUuNSwzLjg2NCwxNS41LDhTMTIuMTM3LDE1LjUsOC4wMDEsMTUuNXoiLz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNOC4wMDEsMUMxMS44NiwxLDE1LDQuMTQxLDE1LDhzLTMuMTM5LDctNi45OTksN0M0LjE0LDE1LDEsMTEuODU5LDEsOFM0LjE0LDEsOC4wMDEsMSBNOC4wMDEsMEMzLjU4MiwwLDAsMy41ODIsMCw4czMuNTgyLDgsOC4wMDEsOEMxMi40MTgsMTYsMTYsMTIuNDE4LDE2LDhTMTIuNDE4LDAsOC4wMDEsMEw4LjAwMSwweiIvPjwvZz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNNi43NDUsMTIuNTg5Yy0wLjIyNywwLjEyMi0wLjQ5NywwLjI0Ny0wLjY4NCwwLjI0N2MtMC4zMTgsMC0wLjUwMS0wLjE2NC0wLjUwMS0wLjQ1MmMwLTAuMjA3LDAuMTQtMC4zNzUsMC41OTUtMC42MjJjMS41NDktMC45MDQsMi41OTQtMi4yNzIsMi41OTQtMy43MjFjMC0wLjgyNS0wLjIyNy0xLjExOS0wLjY4MS0xLjExOWMtMC4xMzUsMC0wLjMyLDAuMjE5LTAuNjM2LDAuMjE5SDcuMTU3QzYuMTAyLDcuMTQzLDUuMzMzLDYuMjY0LDUuMzMzLDUuMjNjMC0xLjE1MiwwLjk1OC0yLjAwNiwyLjI4LTIuMDA2YzEuNzc3LDAsMy4wNTMsMS4zNzMsMy4wNTMsMy40M0MxMC42NjYsOS4yMTUsOS4yMDMsMTEuMjcsNi43NDUsMTIuNTg5Ii8+PC9nPjwvc3ZnPg">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5550307C-79EB-4264-B1AC-FB6B101EA763}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11239500" y="12954000"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="25" name="AutoShape 3" descr="data:image/svg+xml;base64,PD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiPz48IURPQ1RZUEUgc3ZnIFBVQkxJQyAiLS8vVzNDLy9EVEQgU1ZHIDEuMS8vRU4iICJodHRwOi8vd3d3LnczLm9yZy9HcmFwaGljcy9TVkcvMS4xL0RURC9zdmcxMS5kdGQiPjxzdmcgdmVyc2lvbj0iMS4xIiBpZD0iRWJlbmVfMSIgeG1sbnM9Imh0dHA6Ly93d3cudzMub3JnLzIwMDAvc3ZnIiB4bWxuczp4bGluaz0iaHR0cDovL3d3dy53My5vcmcvMTk5OS94bGluayIgeD0iMHB4IiB5PSIwcHgiIHdpZHRoPSIxNnB4IiBoZWlnaHQ9IjE2cHgiIHZpZXdCb3g9IjAgMCAxNiAxNiIgZW5hYmxlLWJhY2tncm91bmQ9Im5ldyAwIDAgMTYgMTYiIHhtbDpzcGFjZT0icHJlc2VydmUiPjxnPjxnPjxwYXRoIGZpbGw9IiNGRkZGRkYiIGQ9Ik04LjAwMSwxNS41QzMuODY0LDE1LjUsMC41LDEyLjEzNiwwLjUsOGMwLTQuMTM1LDMuMzY1LTcuNSw3LjUwMS03LjVTMTUuNSwzLjg2NCwxNS41LDhTMTIuMTM3LDE1LjUsOC4wMDEsMTUuNXoiLz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNOC4wMDEsMUMxMS44NiwxLDE1LDQuMTQxLDE1LDhzLTMuMTM5LDctNi45OTksN0M0LjE0LDE1LDEsMTEuODU5LDEsOFM0LjE0LDEsOC4wMDEsMSBNOC4wMDEsMEMzLjU4MiwwLDAsMy41ODIsMCw4czMuNTgyLDgsOC4wMDEsOEMxMi40MTgsMTYsMTYsMTIuNDE4LDE2LDhTMTIuNDE4LDAsOC4wMDEsMEw4LjAwMSwweiIvPjwvZz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNNi43NDUsMTIuNTg5Yy0wLjIyNywwLjEyMi0wLjQ5NywwLjI0Ny0wLjY4NCwwLjI0N2MtMC4zMTgsMC0wLjUwMS0wLjE2NC0wLjUwMS0wLjQ1MmMwLTAuMjA3LDAuMTQtMC4zNzUsMC41OTUtMC42MjJjMS41NDktMC45MDQsMi41OTQtMi4yNzIsMi41OTQtMy43MjFjMC0wLjgyNS0wLjIyNy0xLjExOS0wLjY4MS0xLjExOWMtMC4xMzUsMC0wLjMyLDAuMjE5LTAuNjM2LDAuMjE5SDcuMTU3QzYuMTAyLDcuMTQzLDUuMzMzLDYuMjY0LDUuMzMzLDUuMjNjMC0xLjE1MiwwLjk1OC0yLjAwNiwyLjI4LTIuMDA2YzEuNzc3LDAsMy4wNTMsMS4zNzMsMy4wNTMsMy40M0MxMC42NjYsOS4yMTUsOS4yMDMsMTEuMjcsNi43NDUsMTIuNTg5Ii8+PC9nPjwvc3ZnPg">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{256AD30F-4EA4-4C31-BF8A-0EB6EC95CEB0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11239500" y="13144500"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="26" name="AutoShape 3" descr="data:image/svg+xml;base64,PD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiPz48IURPQ1RZUEUgc3ZnIFBVQkxJQyAiLS8vVzNDLy9EVEQgU1ZHIDEuMS8vRU4iICJodHRwOi8vd3d3LnczLm9yZy9HcmFwaGljcy9TVkcvMS4xL0RURC9zdmcxMS5kdGQiPjxzdmcgdmVyc2lvbj0iMS4xIiBpZD0iRWJlbmVfMSIgeG1sbnM9Imh0dHA6Ly93d3cudzMub3JnLzIwMDAvc3ZnIiB4bWxuczp4bGluaz0iaHR0cDovL3d3dy53My5vcmcvMTk5OS94bGluayIgeD0iMHB4IiB5PSIwcHgiIHdpZHRoPSIxNnB4IiBoZWlnaHQ9IjE2cHgiIHZpZXdCb3g9IjAgMCAxNiAxNiIgZW5hYmxlLWJhY2tncm91bmQ9Im5ldyAwIDAgMTYgMTYiIHhtbDpzcGFjZT0icHJlc2VydmUiPjxnPjxnPjxwYXRoIGZpbGw9IiNGRkZGRkYiIGQ9Ik04LjAwMSwxNS41QzMuODY0LDE1LjUsMC41LDEyLjEzNiwwLjUsOGMwLTQuMTM1LDMuMzY1LTcuNSw3LjUwMS03LjVTMTUuNSwzLjg2NCwxNS41LDhTMTIuMTM3LDE1LjUsOC4wMDEsMTUuNXoiLz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNOC4wMDEsMUMxMS44NiwxLDE1LDQuMTQxLDE1LDhzLTMuMTM5LDctNi45OTksN0M0LjE0LDE1LDEsMTEuODU5LDEsOFM0LjE0LDEsOC4wMDEsMSBNOC4wMDEsMEMzLjU4MiwwLDAsMy41ODIsMCw4czMuNTgyLDgsOC4wMDEsOEMxMi40MTgsMTYsMTYsMTIuNDE4LDE2LDhTMTIuNDE4LDAsOC4wMDEsMEw4LjAwMSwweiIvPjwvZz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNNi43NDUsMTIuNTg5Yy0wLjIyNywwLjEyMi0wLjQ5NywwLjI0Ny0wLjY4NCwwLjI0N2MtMC4zMTgsMC0wLjUwMS0wLjE2NC0wLjUwMS0wLjQ1MmMwLTAuMjA3LDAuMTQtMC4zNzUsMC41OTUtMC42MjJjMS41NDktMC45MDQsMi41OTQtMi4yNzIsMi41OTQtMy43MjFjMC0wLjgyNS0wLjIyNy0xLjExOS0wLjY4MS0xLjExOWMtMC4xMzUsMC0wLjMyLDAuMjE5LTAuNjM2LDAuMjE5SDcuMTU3QzYuMTAyLDcuMTQzLDUuMzMzLDYuMjY0LDUuMzMzLDUuMjNjMC0xLjE1MiwwLjk1OC0yLjAwNiwyLjI4LTIuMDA2YzEuNzc3LDAsMy4wNTMsMS4zNzMsMy4wNTMsMy40M0MxMC42NjYsOS4yMTUsOS4yMDMsMTEuMjcsNi43NDUsMTIuNTg5Ii8+PC9nPjwvc3ZnPg">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30142F25-DA37-4353-AB88-5BEABC2073EB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11239500" y="13144500"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="304800"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="27" name="AutoShape 3" descr="data:image/svg+xml;base64,PD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiPz48IURPQ1RZUEUgc3ZnIFBVQkxJQyAiLS8vVzNDLy9EVEQgU1ZHIDEuMS8vRU4iICJodHRwOi8vd3d3LnczLm9yZy9HcmFwaGljcy9TVkcvMS4xL0RURC9zdmcxMS5kdGQiPjxzdmcgdmVyc2lvbj0iMS4xIiBpZD0iRWJlbmVfMSIgeG1sbnM9Imh0dHA6Ly93d3cudzMub3JnLzIwMDAvc3ZnIiB4bWxuczp4bGluaz0iaHR0cDovL3d3dy53My5vcmcvMTk5OS94bGluayIgeD0iMHB4IiB5PSIwcHgiIHdpZHRoPSIxNnB4IiBoZWlnaHQ9IjE2cHgiIHZpZXdCb3g9IjAgMCAxNiAxNiIgZW5hYmxlLWJhY2tncm91bmQ9Im5ldyAwIDAgMTYgMTYiIHhtbDpzcGFjZT0icHJlc2VydmUiPjxnPjxnPjxwYXRoIGZpbGw9IiNGRkZGRkYiIGQ9Ik04LjAwMSwxNS41QzMuODY0LDE1LjUsMC41LDEyLjEzNiwwLjUsOGMwLTQuMTM1LDMuMzY1LTcuNSw3LjUwMS03LjVTMTUuNSwzLjg2NCwxNS41LDhTMTIuMTM3LDE1LjUsOC4wMDEsMTUuNXoiLz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNOC4wMDEsMUMxMS44NiwxLDE1LDQuMTQxLDE1LDhzLTMuMTM5LDctNi45OTksN0M0LjE0LDE1LDEsMTEuODU5LDEsOFM0LjE0LDEsOC4wMDEsMSBNOC4wMDEsMEMzLjU4MiwwLDAsMy41ODIsMCw4czMuNTgyLDgsOC4wMDEsOEMxMi40MTgsMTYsMTYsMTIuNDE4LDE2LDhTMTIuNDE4LDAsOC4wMDEsMEw4LjAwMSwweiIvPjwvZz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNNi43NDUsMTIuNTg5Yy0wLjIyNywwLjEyMi0wLjQ5NywwLjI0Ny0wLjY4NCwwLjI0N2MtMC4zMTgsMC0wLjUwMS0wLjE2NC0wLjUwMS0wLjQ1MmMwLTAuMjA3LDAuMTQtMC4zNzUsMC41OTUtMC42MjJjMS41NDktMC45MDQsMi41OTQtMi4yNzIsMi41OTQtMy43MjFjMC0wLjgyNS0wLjIyNy0xLjExOS0wLjY4MS0xLjExOWMtMC4xMzUsMC0wLjMyLDAuMjE5LTAuNjM2LDAuMjE5SDcuMTU3QzYuMTAyLDcuMTQzLDUuMzMzLDYuMjY0LDUuMzMzLDUuMjNjMC0xLjE1MiwwLjk1OC0yLjAwNiwyLjI4LTIuMDA2YzEuNzc3LDAsMy4wNTMsMS4zNzMsMy4wNTMsMy40M0MxMC42NjYsOS4yMTUsOS4yMDMsMTEuMjcsNi43NDUsMTIuNTg5Ii8+PC9nPjwvc3ZnPg">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{17959B61-6AE3-4B1C-8188-9CCA233DD994}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="11239500" y="13144500"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3485,7 +3817,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:AI70"/>
+  <dimension ref="A1:AI71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="31" customWidth="1"/>
@@ -3533,7 +3865,7 @@
         <v>163</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="N1" s="4" t="s">
         <v>164</v>
@@ -3623,20 +3955,20 @@
         <v>2025</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>145</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="10" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>143</v>
@@ -3645,13 +3977,13 @@
         <v>213</v>
       </c>
       <c r="Q2" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="R2" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="R2" s="2" t="s">
-        <v>469</v>
-      </c>
       <c r="S2" s="2" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="T2" s="2"/>
       <c r="U2" s="2"/>
@@ -3705,17 +4037,17 @@
         <v>2022</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>110</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2" t="s">
@@ -3725,13 +4057,13 @@
         <v>202</v>
       </c>
       <c r="Q3" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="R3" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="R3" s="2" t="s">
-        <v>473</v>
-      </c>
       <c r="S3" s="2" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
@@ -3881,7 +4213,7 @@
       </c>
       <c r="K5" s="2"/>
       <c r="L5" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="N5" s="2" t="s">
         <v>320</v>
@@ -3899,7 +4231,7 @@
         <v>319</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
@@ -3961,7 +4293,7 @@
         <v>19</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="K6" s="2"/>
       <c r="N6" s="2"/>
@@ -3972,11 +4304,11 @@
         <v>196</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="R6" s="2"/>
       <c r="S6" s="2" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
@@ -4053,7 +4385,7 @@
         <v>318</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
@@ -4124,11 +4456,11 @@
         <v>209</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="R8" s="2"/>
       <c r="S8" s="2" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="T8" s="2"/>
       <c r="U8" s="2"/>
@@ -4197,11 +4529,11 @@
         <v>216</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="R9" s="2"/>
       <c r="S9" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="T9" s="2"/>
       <c r="U9" s="2"/>
@@ -4259,11 +4591,11 @@
         <v>104</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2" t="s">
@@ -4273,11 +4605,11 @@
         <v>200</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="R10" s="2"/>
       <c r="S10" s="2" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="T10" s="2"/>
       <c r="U10" s="2"/>
@@ -4350,11 +4682,11 @@
         <v>217</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="R11" s="2"/>
       <c r="S11" s="2" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
@@ -4412,11 +4744,11 @@
         <v>19</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="2" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2" t="s">
@@ -4500,7 +4832,7 @@
         <v>204</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
@@ -4543,7 +4875,7 @@
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>335</v>
@@ -4614,7 +4946,7 @@
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>336</v>
@@ -4683,7 +5015,7 @@
     </row>
     <row r="16" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>337</v>
@@ -4762,7 +5094,7 @@
         <v>152</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2" t="s">
@@ -4795,7 +5127,7 @@
         <v>193</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="R17" s="2"/>
       <c r="S17" s="2"/>
@@ -4859,7 +5191,7 @@
       </c>
       <c r="K18" s="2"/>
       <c r="L18" s="2" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2" t="s">
@@ -4869,11 +5201,11 @@
         <v>206</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="R18" s="2"/>
       <c r="S18" s="2" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="T18" s="2"/>
       <c r="U18" s="2"/>
@@ -4935,7 +5267,7 @@
       </c>
       <c r="K19" s="2"/>
       <c r="L19" s="2" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2" t="s">
@@ -4945,7 +5277,7 @@
         <v>189</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="R19" s="2"/>
       <c r="S19" s="2"/>
@@ -5005,7 +5337,7 @@
         <v>14</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="K20" s="2"/>
       <c r="L20" s="2">
@@ -5019,11 +5351,11 @@
         <v>208</v>
       </c>
       <c r="Q20" s="2" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="R20" s="2"/>
       <c r="S20" s="2" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
@@ -5058,7 +5390,7 @@
     </row>
     <row r="21" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>341</v>
@@ -5203,7 +5535,7 @@
     </row>
     <row r="23" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>343</v>
@@ -5382,7 +5714,7 @@
         <v>220</v>
       </c>
       <c r="Q25" s="2" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
@@ -5453,7 +5785,7 @@
         <v>221</v>
       </c>
       <c r="Q26" s="2" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="R26" s="2"/>
       <c r="S26" s="2"/>
@@ -5524,7 +5856,7 @@
         <v>222</v>
       </c>
       <c r="Q27" s="2" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
@@ -5595,7 +5927,7 @@
         <v>223</v>
       </c>
       <c r="Q28" s="2" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="R28" s="2"/>
       <c r="S28" s="2"/>
@@ -5666,7 +5998,7 @@
         <v>211</v>
       </c>
       <c r="Q29" s="2" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
@@ -5737,7 +6069,7 @@
         <v>224</v>
       </c>
       <c r="Q30" s="2" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="R30" s="2"/>
       <c r="S30" s="2"/>
@@ -5786,8 +6118,8 @@
       <c r="E31" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="F31" s="6">
-        <v>45853</v>
+      <c r="F31" s="6" t="s">
+        <v>583</v>
       </c>
       <c r="G31" s="6">
         <v>2025</v>
@@ -5803,7 +6135,7 @@
       </c>
       <c r="K31" s="2"/>
       <c r="L31" s="2" t="s">
-        <v>443</v>
+        <v>584</v>
       </c>
       <c r="N31" s="7" t="s">
         <v>297</v>
@@ -5821,7 +6153,7 @@
         <v>298</v>
       </c>
       <c r="S31" s="2" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="T31" s="2"/>
       <c r="U31" s="2"/>
@@ -5997,7 +6329,7 @@
         <v>314</v>
       </c>
       <c r="S33" s="2" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="T33" s="2"/>
       <c r="U33" s="2"/>
@@ -6419,7 +6751,7 @@
         <v>2020</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>32</v>
@@ -6491,7 +6823,7 @@
         <v>22</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>289</v>
@@ -6710,7 +7042,7 @@
         <v>405</v>
       </c>
       <c r="R41" s="2" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="S41" s="2" t="s">
         <v>427</v>
@@ -6869,7 +7201,7 @@
         <v>19</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="K43" s="2"/>
       <c r="L43" s="2" t="s">
@@ -6891,7 +7223,7 @@
         <v>317</v>
       </c>
       <c r="S43" s="2" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="T43" s="2"/>
       <c r="U43" s="2"/>
@@ -6981,7 +7313,7 @@
         <v>430</v>
       </c>
       <c r="S44" s="2" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="T44" s="2"/>
       <c r="U44" s="2"/>
@@ -7068,7 +7400,7 @@
         <v>408</v>
       </c>
       <c r="R45" s="2" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="S45" s="2" t="s">
         <v>431</v>
@@ -7231,7 +7563,7 @@
       </c>
       <c r="K47" s="2"/>
       <c r="L47" s="2" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2" t="s">
@@ -7241,11 +7573,11 @@
         <v>192</v>
       </c>
       <c r="Q47" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="R47" s="2"/>
       <c r="S47" s="2" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="T47" s="2"/>
       <c r="U47" s="2"/>
@@ -7581,7 +7913,7 @@
       </c>
       <c r="K51" s="2"/>
       <c r="L51" s="2" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="N51" s="2" t="s">
         <v>420</v>
@@ -7597,7 +7929,7 @@
       </c>
       <c r="R51" s="2"/>
       <c r="S51" s="2" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="T51" s="2"/>
       <c r="U51" s="2"/>
@@ -7651,7 +7983,7 @@
         <v>2011</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>72</v>
@@ -7677,7 +8009,7 @@
       </c>
       <c r="R52" s="2"/>
       <c r="S52" s="2" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="T52" s="2"/>
       <c r="U52" s="2"/>
@@ -7739,7 +8071,7 @@
         <v>2024</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="I53" s="2" t="s">
         <v>93</v>
@@ -7752,10 +8084,10 @@
         <v>252</v>
       </c>
       <c r="M53" s="7" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="N53" s="2" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="O53" s="2" t="s">
         <v>95</v>
@@ -7764,7 +8096,7 @@
         <v>197</v>
       </c>
       <c r="Q53" s="2" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="R53" s="2"/>
       <c r="S53" s="2"/>
@@ -7837,10 +8169,10 @@
         <v>248</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="N54" s="2" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="O54" s="2" t="s">
         <v>71</v>
@@ -7849,12 +8181,12 @@
         <v>187</v>
       </c>
       <c r="Q54" s="2" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="R54" s="2"/>
       <c r="S54" s="2"/>
       <c r="T54" s="2" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="U54" s="2"/>
       <c r="V54" s="2"/>
@@ -7922,10 +8254,10 @@
         <v>249</v>
       </c>
       <c r="M55" s="2" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="N55" s="7" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="O55" s="2" t="s">
         <v>79</v>
@@ -7934,7 +8266,7 @@
         <v>190</v>
       </c>
       <c r="Q55" s="2" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="R55" s="2"/>
       <c r="S55" s="2"/>
@@ -8007,7 +8339,7 @@
         <v>250</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" s="2" t="s">
@@ -8017,12 +8349,12 @@
         <v>191</v>
       </c>
       <c r="Q56" s="2" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="R56" s="2"/>
       <c r="S56" s="2"/>
       <c r="T56" s="2" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="U56" s="2"/>
       <c r="V56" s="2"/>
@@ -8081,23 +8413,23 @@
         <v>2015</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="I57" s="2" t="s">
         <v>88</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="K57" s="2"/>
       <c r="L57" s="2" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="N57" s="2" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="O57" s="2" t="s">
         <v>89</v>
@@ -8106,12 +8438,12 @@
         <v>194</v>
       </c>
       <c r="Q57" s="2" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="R57" s="2"/>
       <c r="S57" s="2"/>
       <c r="T57" s="2" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="U57" s="2"/>
       <c r="V57" s="2"/>
@@ -8177,17 +8509,17 @@
         <v>253</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="N58" s="7" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="O58" s="2" t="s">
         <v>127</v>
       </c>
       <c r="P58" s="2"/>
       <c r="Q58" s="7" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="R58" s="2"/>
       <c r="S58" s="2"/>
@@ -8260,10 +8592,10 @@
         <v>247</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="O59" s="2" t="s">
         <v>50</v>
@@ -8272,7 +8604,7 @@
         <v>178</v>
       </c>
       <c r="Q59" s="2" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="R59" s="2"/>
       <c r="S59" s="2"/>
@@ -8314,7 +8646,7 @@
         <v>17</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>289</v>
@@ -8421,7 +8753,7 @@
         <v>15</v>
       </c>
       <c r="N61" s="2" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="O61" s="2" t="s">
         <v>16</v>
@@ -8470,7 +8802,7 @@
         <v>152</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" s="2" t="s">
@@ -8480,13 +8812,13 @@
         <v>155</v>
       </c>
       <c r="F62" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="G62" s="6" t="s">
         <v>529</v>
       </c>
-      <c r="G62" s="6" t="s">
+      <c r="H62" s="2" t="s">
         <v>530</v>
-      </c>
-      <c r="H62" s="2" t="s">
-        <v>531</v>
       </c>
       <c r="I62" s="2"/>
       <c r="J62" s="2" t="s">
@@ -8494,17 +8826,17 @@
       </c>
       <c r="K62" s="2"/>
       <c r="L62" s="2" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
       <c r="P62" s="2"/>
       <c r="Q62" s="2" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="R62" s="2"/>
       <c r="S62" s="2" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="T62" s="2"/>
       <c r="U62" s="2"/>
@@ -8528,7 +8860,7 @@
         <v>152</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" s="2" t="s">
@@ -8538,10 +8870,10 @@
         <v>155</v>
       </c>
       <c r="F63" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="G63" s="6" t="s">
         <v>535</v>
-      </c>
-      <c r="G63" s="6" t="s">
-        <v>536</v>
       </c>
       <c r="H63" s="2" t="s">
         <v>391</v>
@@ -8552,17 +8884,17 @@
       </c>
       <c r="K63" s="2"/>
       <c r="L63" s="2" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
       <c r="P63" s="2"/>
       <c r="Q63" s="2" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="R63" s="2"/>
       <c r="S63" s="2" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="T63" s="2"/>
       <c r="U63" s="2"/>
@@ -8586,7 +8918,7 @@
         <v>152</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" s="2" t="s">
@@ -8596,10 +8928,10 @@
         <v>155</v>
       </c>
       <c r="F64" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="G64" s="6" t="s">
         <v>540</v>
-      </c>
-      <c r="G64" s="6" t="s">
-        <v>541</v>
       </c>
       <c r="H64" s="2" t="s">
         <v>381</v>
@@ -8610,17 +8942,17 @@
       </c>
       <c r="K64" s="2"/>
       <c r="L64" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
       <c r="P64" s="2"/>
       <c r="Q64" s="2" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="R64" s="2"/>
       <c r="S64" s="2" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="T64" s="2"/>
       <c r="U64" s="2"/>
@@ -8644,7 +8976,7 @@
         <v>152</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>289</v>
@@ -8656,27 +8988,27 @@
         <v>155</v>
       </c>
       <c r="F65" s="6" t="s">
+        <v>544</v>
+      </c>
+      <c r="G65" s="6" t="s">
         <v>545</v>
-      </c>
-      <c r="G65" s="6" t="s">
-        <v>546</v>
       </c>
       <c r="H65" s="2" t="s">
         <v>381</v>
       </c>
       <c r="I65" s="2"/>
       <c r="J65" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="K65" s="2"/>
       <c r="L65" s="2" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
       <c r="P65" s="2"/>
       <c r="Q65" s="2" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="R65" s="2"/>
       <c r="S65" s="2"/>
@@ -8702,7 +9034,7 @@
         <v>152</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" s="2" t="s">
@@ -8712,10 +9044,10 @@
         <v>155</v>
       </c>
       <c r="F66" s="6" t="s">
+        <v>550</v>
+      </c>
+      <c r="G66" s="6" t="s">
         <v>551</v>
-      </c>
-      <c r="G66" s="6" t="s">
-        <v>552</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>381</v>
@@ -8726,17 +9058,17 @@
       </c>
       <c r="K66" s="2"/>
       <c r="L66" s="2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="N66" s="2"/>
       <c r="O66" s="2"/>
       <c r="P66" s="2"/>
       <c r="Q66" s="2" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="R66" s="2"/>
       <c r="S66" s="2" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="T66" s="2"/>
       <c r="U66" s="2"/>
@@ -8760,7 +9092,7 @@
         <v>152</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" s="2" t="s">
@@ -8773,28 +9105,28 @@
         <v>268</v>
       </c>
       <c r="G67" s="6" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="H67" s="2" t="s">
         <v>381</v>
       </c>
       <c r="I67" s="2"/>
       <c r="J67" s="8" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="K67" s="2"/>
       <c r="L67" s="8" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="N67" s="2"/>
       <c r="O67" s="2"/>
       <c r="P67" s="2"/>
       <c r="Q67" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="R67" s="2"/>
       <c r="S67" s="2" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="T67" s="2"/>
       <c r="U67" s="2"/>
@@ -8818,7 +9150,7 @@
         <v>152</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" s="2" t="s">
@@ -8828,10 +9160,10 @@
         <v>155</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="H68" s="2" t="s">
         <v>392</v>
@@ -8842,17 +9174,17 @@
       </c>
       <c r="K68" s="2"/>
       <c r="L68" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
       <c r="P68" s="2"/>
       <c r="Q68" s="2" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="R68" s="2"/>
       <c r="S68" s="2" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="T68" s="2"/>
       <c r="U68" s="2"/>
@@ -8876,7 +9208,7 @@
         <v>152</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" s="2" t="s">
@@ -8886,10 +9218,10 @@
         <v>155</v>
       </c>
       <c r="F69" s="6" t="s">
+        <v>564</v>
+      </c>
+      <c r="G69" s="6" t="s">
         <v>565</v>
-      </c>
-      <c r="G69" s="6" t="s">
-        <v>566</v>
       </c>
       <c r="H69" s="2" t="s">
         <v>381</v>
@@ -8900,17 +9232,17 @@
       </c>
       <c r="K69" s="2"/>
       <c r="L69" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
       <c r="P69" s="2"/>
       <c r="Q69" s="9" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="R69" s="2"/>
       <c r="S69" s="2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="T69" s="2"/>
       <c r="U69" s="2"/>
@@ -8934,7 +9266,7 @@
         <v>152</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" s="2" t="s">
@@ -8944,13 +9276,13 @@
         <v>155</v>
       </c>
       <c r="F70" s="6" t="s">
+        <v>570</v>
+      </c>
+      <c r="G70" s="6" t="s">
         <v>571</v>
       </c>
-      <c r="G70" s="6" t="s">
+      <c r="H70" s="2" t="s">
         <v>572</v>
-      </c>
-      <c r="H70" s="2" t="s">
-        <v>573</v>
       </c>
       <c r="I70" s="2"/>
       <c r="J70" s="2" t="s">
@@ -8958,17 +9290,17 @@
       </c>
       <c r="K70" s="2"/>
       <c r="L70" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="N70" s="2"/>
       <c r="O70" s="2"/>
       <c r="P70" s="2"/>
       <c r="Q70" s="2" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="R70" s="2"/>
       <c r="S70" s="2" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="T70" s="2"/>
       <c r="U70" s="2"/>
@@ -8987,6 +9319,64 @@
       <c r="AH70" s="2"/>
       <c r="AI70" s="2"/>
     </row>
+    <row r="71" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="C71" s="2"/>
+      <c r="D71" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>585</v>
+      </c>
+      <c r="G71" s="6" t="s">
+        <v>586</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="I71" s="2"/>
+      <c r="J71" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="K71" s="2"/>
+      <c r="L71" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="N71" s="2"/>
+      <c r="O71" s="2"/>
+      <c r="P71" s="2"/>
+      <c r="Q71" s="2" t="s">
+        <v>589</v>
+      </c>
+      <c r="R71" s="2"/>
+      <c r="S71" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="T71" s="2"/>
+      <c r="U71" s="2"/>
+      <c r="V71" s="2"/>
+      <c r="W71" s="2"/>
+      <c r="X71" s="2"/>
+      <c r="Y71" s="2"/>
+      <c r="Z71" s="2"/>
+      <c r="AA71" s="2"/>
+      <c r="AB71" s="2"/>
+      <c r="AC71" s="2"/>
+      <c r="AD71" s="2"/>
+      <c r="AE71" s="2"/>
+      <c r="AF71" s="2"/>
+      <c r="AG71" s="2"/>
+      <c r="AH71" s="2"/>
+      <c r="AI71" s="2"/>
+    </row>
   </sheetData>
   <sortState ref="A2:AI61">
     <sortCondition descending="1" ref="A2:A61"/>

</xml_diff>

<commit_message>
Update upon Governance Publication (pubs, data and data viz, CV, blog)
</commit_message>
<xml_diff>
--- a/files/CR_Publications.xlsx
+++ b/files/CR_Publications.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rauh\NextCloudSync\WZB_CR\Datensaetze\ChRauh.github.io\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WZB-Nextcloud\WZB_CR\Datensaetze\ChRauh.github.io\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75E1DBCB-2C45-4822-A3FC-2A39C0121464}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3291414-F351-4F2D-A6F2-B40C7D7434A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GS-profile_20250821" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="601">
   <si>
     <t>Cites</t>
   </si>
@@ -1796,6 +1796,33 @@
   </si>
   <si>
     <t>**Zwischen Wirtschaft und Werten: Zum Selbst- und Fremdbild der Europäischen Union in der internationalen Ordnung**</t>
+  </si>
+  <si>
+    <t>**Responsive to What? Explaining the Information Quality of Public Comments on Bureaucratic Policymaking Using a Text-as-Data Approach**</t>
+  </si>
+  <si>
+    <t>Adriana Bunea, Sergiu Lipcean, &lt;u&gt;Christian Rauh&lt;/u&gt;</t>
+  </si>
+  <si>
+    <t>Governance</t>
+  </si>
+  <si>
+    <t>10.1111/gove.70122</t>
+  </si>
+  <si>
+    <t>https://onlinelibrary.wiley.com/doi/10.1111/gove.70122</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.7910/DVN/M606UR</t>
+  </si>
+  <si>
+    <t>https://onlinelibrary.wiley.com/doi/epdf/10.1111/gove.70122</t>
+  </si>
+  <si>
+    <t>2026-03-27</t>
+  </si>
+  <si>
+    <t>Online First</t>
   </si>
 </sst>
 </file>
@@ -2288,7 +2315,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2302,10 +2329,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="42" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -3395,98 +3419,9 @@
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="25" name="AutoShape 3" descr="data:image/svg+xml;base64,PD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiPz48IURPQ1RZUEUgc3ZnIFBVQkxJQyAiLS8vVzNDLy9EVEQgU1ZHIDEuMS8vRU4iICJodHRwOi8vd3d3LnczLm9yZy9HcmFwaGljcy9TVkcvMS4xL0RURC9zdmcxMS5kdGQiPjxzdmcgdmVyc2lvbj0iMS4xIiBpZD0iRWJlbmVfMSIgeG1sbnM9Imh0dHA6Ly93d3cudzMub3JnLzIwMDAvc3ZnIiB4bWxuczp4bGluaz0iaHR0cDovL3d3dy53My5vcmcvMTk5OS94bGluayIgeD0iMHB4IiB5PSIwcHgiIHdpZHRoPSIxNnB4IiBoZWlnaHQ9IjE2cHgiIHZpZXdCb3g9IjAgMCAxNiAxNiIgZW5hYmxlLWJhY2tncm91bmQ9Im5ldyAwIDAgMTYgMTYiIHhtbDpzcGFjZT0icHJlc2VydmUiPjxnPjxnPjxwYXRoIGZpbGw9IiNGRkZGRkYiIGQ9Ik04LjAwMSwxNS41QzMuODY0LDE1LjUsMC41LDEyLjEzNiwwLjUsOGMwLTQuMTM1LDMuMzY1LTcuNSw3LjUwMS03LjVTMTUuNSwzLjg2NCwxNS41LDhTMTIuMTM3LDE1LjUsOC4wMDEsMTUuNXoiLz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNOC4wMDEsMUMxMS44NiwxLDE1LDQuMTQxLDE1LDhzLTMuMTM5LDctNi45OTksN0M0LjE0LDE1LDEsMTEuODU5LDEsOFM0LjE0LDEsOC4wMDEsMSBNOC4wMDEsMEMzLjU4MiwwLDAsMy41ODIsMCw4czMuNTgyLDgsOC4wMDEsOEMxMi40MTgsMTYsMTYsMTIuNDE4LDE2LDhTMTIuNDE4LDAsOC4wMDEsMEw4LjAwMSwweiIvPjwvZz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNNi43NDUsMTIuNTg5Yy0wLjIyNywwLjEyMi0wLjQ5NywwLjI0Ny0wLjY4NCwwLjI0N2MtMC4zMTgsMC0wLjUwMS0wLjE2NC0wLjUwMS0wLjQ1MmMwLTAuMjA3LDAuMTQtMC4zNzUsMC41OTUtMC42MjJjMS41NDktMC45MDQsMi41OTQtMi4yNzIsMi41OTQtMy43MjFjMC0wLjgyNS0wLjIyNy0xLjExOS0wLjY4MS0xLjExOWMtMC4xMzUsMC0wLjMyLDAuMjE5LTAuNjM2LDAuMjE5SDcuMTU3QzYuMTAyLDcuMTQzLDUuMzMzLDYuMjY0LDUuMzMzLDUuMjNjMC0xLjE1MiwwLjk1OC0yLjAwNiwyLjI4LTIuMDA2YzEuNzc3LDAsMy4wNTMsMS4zNzMsMy4wNTMsMy40M0MxMC42NjYsOS4yMTUsOS4yMDMsMTEuMjcsNi43NDUsMTIuNTg5Ii8+PC9nPjwvc3ZnPg">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{256AD30F-4EA4-4C31-BF8A-0EB6EC95CEB0}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="11239500" y="13144500"/>
-          <a:ext cx="304800" cy="304800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>70</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="304800" cy="304800"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="26" name="AutoShape 3" descr="data:image/svg+xml;base64,PD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiPz48IURPQ1RZUEUgc3ZnIFBVQkxJQyAiLS8vVzNDLy9EVEQgU1ZHIDEuMS8vRU4iICJodHRwOi8vd3d3LnczLm9yZy9HcmFwaGljcy9TVkcvMS4xL0RURC9zdmcxMS5kdGQiPjxzdmcgdmVyc2lvbj0iMS4xIiBpZD0iRWJlbmVfMSIgeG1sbnM9Imh0dHA6Ly93d3cudzMub3JnLzIwMDAvc3ZnIiB4bWxuczp4bGluaz0iaHR0cDovL3d3dy53My5vcmcvMTk5OS94bGluayIgeD0iMHB4IiB5PSIwcHgiIHdpZHRoPSIxNnB4IiBoZWlnaHQ9IjE2cHgiIHZpZXdCb3g9IjAgMCAxNiAxNiIgZW5hYmxlLWJhY2tncm91bmQ9Im5ldyAwIDAgMTYgMTYiIHhtbDpzcGFjZT0icHJlc2VydmUiPjxnPjxnPjxwYXRoIGZpbGw9IiNGRkZGRkYiIGQ9Ik04LjAwMSwxNS41QzMuODY0LDE1LjUsMC41LDEyLjEzNiwwLjUsOGMwLTQuMTM1LDMuMzY1LTcuNSw3LjUwMS03LjVTMTUuNSwzLjg2NCwxNS41LDhTMTIuMTM3LDE1LjUsOC4wMDEsMTUuNXoiLz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNOC4wMDEsMUMxMS44NiwxLDE1LDQuMTQxLDE1LDhzLTMuMTM5LDctNi45OTksN0M0LjE0LDE1LDEsMTEuODU5LDEsOFM0LjE0LDEsOC4wMDEsMSBNOC4wMDEsMEMzLjU4MiwwLDAsMy41ODIsMCw4czMuNTgyLDgsOC4wMDEsOEMxMi40MTgsMTYsMTYsMTIuNDE4LDE2LDhTMTIuNDE4LDAsOC4wMDEsMEw4LjAwMSwweiIvPjwvZz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNNi43NDUsMTIuNTg5Yy0wLjIyNywwLjEyMi0wLjQ5NywwLjI0Ny0wLjY4NCwwLjI0N2MtMC4zMTgsMC0wLjUwMS0wLjE2NC0wLjUwMS0wLjQ1MmMwLTAuMjA3LDAuMTQtMC4zNzUsMC41OTUtMC42MjJjMS41NDktMC45MDQsMi41OTQtMi4yNzIsMi41OTQtMy43MjFjMC0wLjgyNS0wLjIyNy0xLjExOS0wLjY4MS0xLjExOWMtMC4xMzUsMC0wLjMyLDAuMjE5LTAuNjM2LDAuMjE5SDcuMTU3QzYuMTAyLDcuMTQzLDUuMzMzLDYuMjY0LDUuMzMzLDUuMjNjMC0xLjE1MiwwLjk1OC0yLjAwNiwyLjI4LTIuMDA2YzEuNzc3LDAsMy4wNTMsMS4zNzMsMy4wNTMsMy40M0MxMC42NjYsOS4yMTUsOS4yMDMsMTEuMjcsNi43NDUsMTIuNTg5Ii8+PC9nPjwvc3ZnPg">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30142F25-DA37-4353-AB88-5BEABC2073EB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="11239500" y="13144500"/>
-          <a:ext cx="304800" cy="304800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>70</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="304800" cy="304800"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="27" name="AutoShape 3" descr="data:image/svg+xml;base64,PD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXRmLTgiPz48IURPQ1RZUEUgc3ZnIFBVQkxJQyAiLS8vVzNDLy9EVEQgU1ZHIDEuMS8vRU4iICJodHRwOi8vd3d3LnczLm9yZy9HcmFwaGljcy9TVkcvMS4xL0RURC9zdmcxMS5kdGQiPjxzdmcgdmVyc2lvbj0iMS4xIiBpZD0iRWJlbmVfMSIgeG1sbnM9Imh0dHA6Ly93d3cudzMub3JnLzIwMDAvc3ZnIiB4bWxuczp4bGluaz0iaHR0cDovL3d3dy53My5vcmcvMTk5OS94bGluayIgeD0iMHB4IiB5PSIwcHgiIHdpZHRoPSIxNnB4IiBoZWlnaHQ9IjE2cHgiIHZpZXdCb3g9IjAgMCAxNiAxNiIgZW5hYmxlLWJhY2tncm91bmQ9Im5ldyAwIDAgMTYgMTYiIHhtbDpzcGFjZT0icHJlc2VydmUiPjxnPjxnPjxwYXRoIGZpbGw9IiNGRkZGRkYiIGQ9Ik04LjAwMSwxNS41QzMuODY0LDE1LjUsMC41LDEyLjEzNiwwLjUsOGMwLTQuMTM1LDMuMzY1LTcuNSw3LjUwMS03LjVTMTUuNSwzLjg2NCwxNS41LDhTMTIuMTM3LDE1LjUsOC4wMDEsMTUuNXoiLz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNOC4wMDEsMUMxMS44NiwxLDE1LDQuMTQxLDE1LDhzLTMuMTM5LDctNi45OTksN0M0LjE0LDE1LDEsMTEuODU5LDEsOFM0LjE0LDEsOC4wMDEsMSBNOC4wMDEsMEMzLjU4MiwwLDAsMy41ODIsMCw4czMuNTgyLDgsOC4wMDEsOEMxMi40MTgsMTYsMTYsMTIuNDE4LDE2LDhTMTIuNDE4LDAsOC4wMDEsMEw4LjAwMSwweiIvPjwvZz48cGF0aCBmaWxsPSIjRDUyQjFFIiBkPSJNNi43NDUsMTIuNTg5Yy0wLjIyNywwLjEyMi0wLjQ5NywwLjI0Ny0wLjY4NCwwLjI0N2MtMC4zMTgsMC0wLjUwMS0wLjE2NC0wLjUwMS0wLjQ1MmMwLTAuMjA3LDAuMTQtMC4zNzUsMC41OTUtMC42MjJjMS41NDktMC45MDQsMi41OTQtMi4yNzIsMi41OTQtMy43MjFjMC0wLjgyNS0wLjIyNy0xLjExOS0wLjY4MS0xLjExOWMtMC4xMzUsMC0wLjMyLDAuMjE5LTAuNjM2LDAuMjE5SDcuMTU3QzYuMTAyLDcuMTQzLDUuMzMzLDYuMjY0LDUuMzMzLDUuMjNjMC0xLjE1MiwwLjk1OC0yLjAwNiwyLjI4LTIuMDA2YzEuNzc3LDAsMy4wNTMsMS4zNzMsMy4wNTMsMy40M0MxMC42NjYsOS4yMTUsOS4yMDMsMTEuMjcsNi43NDUsMTIuNTg5Ii8+PC9nPjwvc3ZnPg">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{17959B61-6AE3-4B1C-8188-9CCA233DD994}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3520,9 +3455,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3560,7 +3495,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3666,7 +3601,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3808,7 +3743,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3817,17 +3752,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Tabelle1"/>
-  <dimension ref="A1:AI71"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AI72"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="31" customWidth="1"/>
-    <col min="6" max="7" width="11.5703125" style="1"/>
-    <col min="8" max="8" width="11.42578125" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" style="2"/>
-    <col min="13" max="13" width="11.42578125" style="2"/>
+    <col min="6" max="7" width="11.54296875" style="1"/>
+    <col min="8" max="8" width="11.453125" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" style="2"/>
+    <col min="13" max="13" width="11.453125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>151</v>
       </c>
@@ -3934,7 +3869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>152</v>
       </c>
@@ -3964,7 +3899,7 @@
         <v>466</v>
       </c>
       <c r="K2" s="2"/>
-      <c r="L2" s="10" t="s">
+      <c r="L2" t="s">
         <v>580</v>
       </c>
       <c r="N2" s="2" t="s">
@@ -4016,7 +3951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>152</v>
       </c>
@@ -4094,7 +4029,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>152</v>
       </c>
@@ -4182,7 +4117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>152</v>
       </c>
@@ -4266,7 +4201,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>152</v>
       </c>
@@ -4339,7 +4274,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>152</v>
       </c>
@@ -4418,7 +4353,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>152</v>
       </c>
@@ -4491,7 +4426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>152</v>
       </c>
@@ -4564,7 +4499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>152</v>
       </c>
@@ -4644,7 +4579,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>152</v>
       </c>
@@ -4717,7 +4652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>152</v>
       </c>
@@ -4791,7 +4726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>152</v>
       </c>
@@ -4873,7 +4808,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>486</v>
       </c>
@@ -4944,7 +4879,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>486</v>
       </c>
@@ -5013,7 +4948,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>488</v>
       </c>
@@ -5089,7 +5024,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>152</v>
       </c>
@@ -5160,7 +5095,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>152</v>
       </c>
@@ -5236,7 +5171,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>152</v>
       </c>
@@ -5310,7 +5245,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>152</v>
       </c>
@@ -5388,7 +5323,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>488</v>
       </c>
@@ -5455,7 +5390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>152</v>
       </c>
@@ -5533,7 +5468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>488</v>
       </c>
@@ -5609,7 +5544,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>152</v>
       </c>
@@ -5676,7 +5611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>152</v>
       </c>
@@ -5747,7 +5682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>152</v>
       </c>
@@ -5818,7 +5753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>152</v>
       </c>
@@ -5889,7 +5824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>152</v>
       </c>
@@ -5960,7 +5895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>152</v>
       </c>
@@ -6031,7 +5966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>152</v>
       </c>
@@ -6102,7 +6037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>22</v>
       </c>
@@ -6137,7 +6072,7 @@
       <c r="L31" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="N31" s="7" t="s">
+      <c r="N31" s="2" t="s">
         <v>297</v>
       </c>
       <c r="O31" s="2" t="s">
@@ -6188,7 +6123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>22</v>
       </c>
@@ -6223,7 +6158,7 @@
       <c r="L32" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="N32" s="7" t="s">
+      <c r="N32" s="2" t="s">
         <v>263</v>
       </c>
       <c r="O32" s="2" t="s">
@@ -6278,7 +6213,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>22</v>
       </c>
@@ -6313,7 +6248,7 @@
       <c r="L33" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="N33" s="7" t="s">
+      <c r="N33" s="2" t="s">
         <v>261</v>
       </c>
       <c r="O33" s="2" t="s">
@@ -6368,7 +6303,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>22</v>
       </c>
@@ -6412,7 +6347,7 @@
       <c r="P34" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="Q34" s="7" t="s">
+      <c r="Q34" s="2" t="s">
         <v>299</v>
       </c>
       <c r="R34" s="2" t="s">
@@ -6458,7 +6393,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>22</v>
       </c>
@@ -6493,7 +6428,7 @@
       <c r="L35" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="N35" s="7" t="s">
+      <c r="N35" s="2" t="s">
         <v>304</v>
       </c>
       <c r="O35" s="2" t="s">
@@ -6548,7 +6483,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>22</v>
       </c>
@@ -6583,7 +6518,7 @@
       <c r="L36" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="N36" s="7" t="s">
+      <c r="N36" s="2" t="s">
         <v>308</v>
       </c>
       <c r="O36" s="2" t="s">
@@ -6638,7 +6573,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>22</v>
       </c>
@@ -6673,7 +6608,7 @@
       <c r="L37" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="N37" s="7" t="s">
+      <c r="N37" s="2" t="s">
         <v>312</v>
       </c>
       <c r="O37" s="2" t="s">
@@ -6728,7 +6663,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="38" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>22</v>
       </c>
@@ -6775,7 +6710,7 @@
       <c r="Q38" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="R38" s="7" t="s">
+      <c r="R38" s="2" t="s">
         <v>316</v>
       </c>
       <c r="S38" s="2" t="s">
@@ -6818,7 +6753,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>22</v>
       </c>
@@ -6908,7 +6843,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="40" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>22</v>
       </c>
@@ -6994,7 +6929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>22</v>
       </c>
@@ -7084,7 +7019,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>22</v>
       </c>
@@ -7128,7 +7063,7 @@
       <c r="P42" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="Q42" s="7" t="s">
+      <c r="Q42" s="2" t="s">
         <v>406</v>
       </c>
       <c r="R42" s="2"/>
@@ -7172,7 +7107,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="43" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>22</v>
       </c>
@@ -7216,7 +7151,7 @@
       <c r="P43" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="Q43" s="7" t="s">
+      <c r="Q43" s="2" t="s">
         <v>403</v>
       </c>
       <c r="R43" s="2" t="s">
@@ -7262,7 +7197,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="44" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>22</v>
       </c>
@@ -7352,7 +7287,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>22</v>
       </c>
@@ -7387,7 +7322,7 @@
       <c r="L45" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="N45" s="7" t="s">
+      <c r="N45" s="2" t="s">
         <v>432</v>
       </c>
       <c r="O45" s="2" t="s">
@@ -7442,7 +7377,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>22</v>
       </c>
@@ -7486,7 +7421,7 @@
       <c r="P46" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="Q46" s="7" t="s">
+      <c r="Q46" s="2" t="s">
         <v>409</v>
       </c>
       <c r="R46" s="2"/>
@@ -7530,7 +7465,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>22</v>
       </c>
@@ -7612,7 +7547,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>22</v>
       </c>
@@ -7702,7 +7637,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="49" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>22</v>
       </c>
@@ -7792,7 +7727,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>22</v>
       </c>
@@ -7827,7 +7762,7 @@
       <c r="L50" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="N50" s="7" t="s">
+      <c r="N50" s="2" t="s">
         <v>442</v>
       </c>
       <c r="O50" s="2" t="s">
@@ -7880,7 +7815,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>22</v>
       </c>
@@ -7960,7 +7895,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="52" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>22</v>
       </c>
@@ -8048,7 +7983,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
@@ -8083,7 +8018,7 @@
       <c r="L53" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="M53" s="7" t="s">
+      <c r="M53" s="2" t="s">
         <v>520</v>
       </c>
       <c r="N53" s="2" t="s">
@@ -8133,7 +8068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>51</v>
       </c>
@@ -8220,7 +8155,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="55" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>51</v>
       </c>
@@ -8256,7 +8191,7 @@
       <c r="M55" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="N55" s="7" t="s">
+      <c r="N55" s="2" t="s">
         <v>478</v>
       </c>
       <c r="O55" s="2" t="s">
@@ -8303,7 +8238,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>51</v>
       </c>
@@ -8390,7 +8325,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>51</v>
       </c>
@@ -8473,7 +8408,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="58" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>51</v>
       </c>
@@ -8511,14 +8446,14 @@
       <c r="M58" s="2" t="s">
         <v>525</v>
       </c>
-      <c r="N58" s="7" t="s">
+      <c r="N58" s="2" t="s">
         <v>479</v>
       </c>
       <c r="O58" s="2" t="s">
         <v>127</v>
       </c>
       <c r="P58" s="2"/>
-      <c r="Q58" s="7" t="s">
+      <c r="Q58" s="2" t="s">
         <v>459</v>
       </c>
       <c r="R58" s="2"/>
@@ -8556,7 +8491,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>51</v>
       </c>
@@ -8641,7 +8576,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="60" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>17</v>
       </c>
@@ -8718,7 +8653,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="61" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>17</v>
       </c>
@@ -8758,18 +8693,18 @@
       <c r="O61" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="P61" s="7" t="s">
+      <c r="P61" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="Q61" s="7" t="s">
+      <c r="Q61" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="R61" s="7"/>
-      <c r="S61" s="7"/>
-      <c r="T61" s="7" t="s">
+      <c r="R61" s="2"/>
+      <c r="S61" s="2"/>
+      <c r="T61" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="U61" s="7"/>
+      <c r="U61" s="2"/>
       <c r="V61" s="2"/>
       <c r="W61" s="2"/>
       <c r="X61" s="2"/>
@@ -8797,7 +8732,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="62" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>152</v>
       </c>
@@ -8855,7 +8790,7 @@
       <c r="AH62" s="2"/>
       <c r="AI62" s="2"/>
     </row>
-    <row r="63" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>152</v>
       </c>
@@ -8913,7 +8848,7 @@
       <c r="AH63" s="2"/>
       <c r="AI63" s="2"/>
     </row>
-    <row r="64" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>152</v>
       </c>
@@ -8971,7 +8906,7 @@
       <c r="AH64" s="2"/>
       <c r="AI64" s="2"/>
     </row>
-    <row r="65" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>152</v>
       </c>
@@ -9029,7 +8964,7 @@
       <c r="AH65" s="2"/>
       <c r="AI65" s="2"/>
     </row>
-    <row r="66" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>152</v>
       </c>
@@ -9087,7 +9022,7 @@
       <c r="AH66" s="2"/>
       <c r="AI66" s="2"/>
     </row>
-    <row r="67" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>152</v>
       </c>
@@ -9111,11 +9046,11 @@
         <v>381</v>
       </c>
       <c r="I67" s="2"/>
-      <c r="J67" s="8" t="s">
+      <c r="J67" t="s">
         <v>555</v>
       </c>
       <c r="K67" s="2"/>
-      <c r="L67" s="8" t="s">
+      <c r="L67" t="s">
         <v>556</v>
       </c>
       <c r="N67" s="2"/>
@@ -9145,7 +9080,7 @@
       <c r="AH67" s="2"/>
       <c r="AI67" s="2"/>
     </row>
-    <row r="68" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>152</v>
       </c>
@@ -9203,7 +9138,7 @@
       <c r="AH68" s="2"/>
       <c r="AI68" s="2"/>
     </row>
-    <row r="69" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>152</v>
       </c>
@@ -9237,7 +9172,7 @@
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
       <c r="P69" s="2"/>
-      <c r="Q69" s="9" t="s">
+      <c r="Q69" s="7" t="s">
         <v>568</v>
       </c>
       <c r="R69" s="2"/>
@@ -9261,7 +9196,7 @@
       <c r="AH69" s="2"/>
       <c r="AI69" s="2"/>
     </row>
-    <row r="70" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>152</v>
       </c>
@@ -9319,7 +9254,7 @@
       <c r="AH70" s="2"/>
       <c r="AI70" s="2"/>
     </row>
-    <row r="71" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>152</v>
       </c>
@@ -9377,8 +9312,53 @@
       <c r="AH71" s="2"/>
       <c r="AI71" s="2"/>
     </row>
+    <row r="72" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="A72" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B72" t="s">
+        <v>592</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E72" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="G72" s="1">
+        <v>2026</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="J72" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="N72" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="O72" s="2"/>
+      <c r="Q72" t="s">
+        <v>596</v>
+      </c>
+      <c r="R72" t="s">
+        <v>597</v>
+      </c>
+      <c r="S72" t="s">
+        <v>598</v>
+      </c>
+      <c r="Y72" t="s">
+        <v>600</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState ref="A2:AI61">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AI61">
     <sortCondition descending="1" ref="A2:A61"/>
     <sortCondition descending="1" ref="F2:F61"/>
   </sortState>

</xml_diff>

<commit_message>
Teaching SS 2026 update (and fixed blog links)
</commit_message>
<xml_diff>
--- a/files/CR_Publications.xlsx
+++ b/files/CR_Publications.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WZB-Nextcloud\WZB_CR\Datensaetze\ChRauh.github.io\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rauh\NextCloudSync\WZB_CR\Datensaetze\ChRauh.github.io\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3291414-F351-4F2D-A6F2-B40C7D7434A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C974637-98F0-4CE0-B56F-5189E91C42AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GS-profile_20250821" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="601">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="602">
   <si>
     <t>Cites</t>
   </si>
@@ -1823,6 +1823,9 @@
   </si>
   <si>
     <t>Online First</t>
+  </si>
+  <si>
+    <t>OU6Ihb5iCvQC</t>
   </si>
 </sst>
 </file>
@@ -3753,16 +3756,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Tabelle1"/>
   <dimension ref="A1:AI72"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="31" customWidth="1"/>
-    <col min="6" max="7" width="11.54296875" style="1"/>
-    <col min="8" max="8" width="11.453125" customWidth="1"/>
-    <col min="12" max="12" width="11.54296875" style="2"/>
-    <col min="13" max="13" width="11.453125" style="2"/>
+    <col min="6" max="7" width="11.5703125" style="1"/>
+    <col min="8" max="8" width="11.42578125" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" style="2"/>
+    <col min="13" max="13" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" s="3" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>151</v>
       </c>
@@ -3869,7 +3872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>152</v>
       </c>
@@ -3951,7 +3954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>152</v>
       </c>
@@ -4029,7 +4032,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>152</v>
       </c>
@@ -4117,7 +4120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>152</v>
       </c>
@@ -4201,7 +4204,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>152</v>
       </c>
@@ -4274,7 +4277,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>152</v>
       </c>
@@ -4353,7 +4356,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>152</v>
       </c>
@@ -4426,7 +4429,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>152</v>
       </c>
@@ -4499,7 +4502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>152</v>
       </c>
@@ -4579,7 +4582,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>152</v>
       </c>
@@ -4652,7 +4655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>152</v>
       </c>
@@ -4726,7 +4729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>152</v>
       </c>
@@ -4808,7 +4811,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>486</v>
       </c>
@@ -4879,7 +4882,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>486</v>
       </c>
@@ -4948,7 +4951,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>488</v>
       </c>
@@ -5024,7 +5027,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>152</v>
       </c>
@@ -5095,7 +5098,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>152</v>
       </c>
@@ -5171,7 +5174,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>152</v>
       </c>
@@ -5245,7 +5248,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>152</v>
       </c>
@@ -5323,7 +5326,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>488</v>
       </c>
@@ -5390,7 +5393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>152</v>
       </c>
@@ -5468,7 +5471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>488</v>
       </c>
@@ -5544,7 +5547,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>152</v>
       </c>
@@ -5611,7 +5614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>152</v>
       </c>
@@ -5682,7 +5685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>152</v>
       </c>
@@ -5753,7 +5756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>152</v>
       </c>
@@ -5824,7 +5827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>152</v>
       </c>
@@ -5895,7 +5898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>152</v>
       </c>
@@ -5966,7 +5969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>152</v>
       </c>
@@ -6037,7 +6040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>22</v>
       </c>
@@ -6123,7 +6126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>22</v>
       </c>
@@ -6213,7 +6216,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="33" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>22</v>
       </c>
@@ -6303,7 +6306,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>22</v>
       </c>
@@ -6393,7 +6396,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="35" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>22</v>
       </c>
@@ -6483,7 +6486,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="36" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>22</v>
       </c>
@@ -6573,7 +6576,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>22</v>
       </c>
@@ -6663,7 +6666,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="38" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>22</v>
       </c>
@@ -6753,7 +6756,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="39" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>22</v>
       </c>
@@ -6843,7 +6846,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="40" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>22</v>
       </c>
@@ -6929,7 +6932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>22</v>
       </c>
@@ -7019,7 +7022,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="42" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>22</v>
       </c>
@@ -7107,7 +7110,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="43" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>22</v>
       </c>
@@ -7197,7 +7200,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="44" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>22</v>
       </c>
@@ -7287,7 +7290,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="45" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>22</v>
       </c>
@@ -7377,7 +7380,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>22</v>
       </c>
@@ -7465,7 +7468,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>22</v>
       </c>
@@ -7547,7 +7550,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>22</v>
       </c>
@@ -7637,7 +7640,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="49" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>22</v>
       </c>
@@ -7727,7 +7730,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>22</v>
       </c>
@@ -7815,7 +7818,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>22</v>
       </c>
@@ -7895,7 +7898,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="52" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>22</v>
       </c>
@@ -7983,7 +7986,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
@@ -8068,7 +8071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>51</v>
       </c>
@@ -8155,7 +8158,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="55" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>51</v>
       </c>
@@ -8238,7 +8241,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>51</v>
       </c>
@@ -8325,7 +8328,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>51</v>
       </c>
@@ -8408,7 +8411,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="58" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>51</v>
       </c>
@@ -8491,7 +8494,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>51</v>
       </c>
@@ -8576,7 +8579,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="60" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>17</v>
       </c>
@@ -8653,7 +8656,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="61" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>17</v>
       </c>
@@ -8732,7 +8735,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="62" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>152</v>
       </c>
@@ -8790,7 +8793,7 @@
       <c r="AH62" s="2"/>
       <c r="AI62" s="2"/>
     </row>
-    <row r="63" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>152</v>
       </c>
@@ -8848,7 +8851,7 @@
       <c r="AH63" s="2"/>
       <c r="AI63" s="2"/>
     </row>
-    <row r="64" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>152</v>
       </c>
@@ -8906,7 +8909,7 @@
       <c r="AH64" s="2"/>
       <c r="AI64" s="2"/>
     </row>
-    <row r="65" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>152</v>
       </c>
@@ -8964,7 +8967,7 @@
       <c r="AH65" s="2"/>
       <c r="AI65" s="2"/>
     </row>
-    <row r="66" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>152</v>
       </c>
@@ -9022,7 +9025,7 @@
       <c r="AH66" s="2"/>
       <c r="AI66" s="2"/>
     </row>
-    <row r="67" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>152</v>
       </c>
@@ -9080,7 +9083,7 @@
       <c r="AH67" s="2"/>
       <c r="AI67" s="2"/>
     </row>
-    <row r="68" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>152</v>
       </c>
@@ -9138,7 +9141,7 @@
       <c r="AH68" s="2"/>
       <c r="AI68" s="2"/>
     </row>
-    <row r="69" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>152</v>
       </c>
@@ -9196,7 +9199,7 @@
       <c r="AH69" s="2"/>
       <c r="AI69" s="2"/>
     </row>
-    <row r="70" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>152</v>
       </c>
@@ -9254,7 +9257,7 @@
       <c r="AH70" s="2"/>
       <c r="AI70" s="2"/>
     </row>
-    <row r="71" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>152</v>
       </c>
@@ -9312,7 +9315,7 @@
       <c r="AH71" s="2"/>
       <c r="AI71" s="2"/>
     </row>
-    <row r="72" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>22</v>
       </c>
@@ -9344,6 +9347,9 @@
         <v>595</v>
       </c>
       <c r="O72" s="2"/>
+      <c r="P72" t="s">
+        <v>601</v>
+      </c>
       <c r="Q72" t="s">
         <v>596</v>
       </c>

</xml_diff>